<commit_message>
data: archive run 2026-06-20T19:19:08Z
</commit_message>
<xml_diff>
--- a/archive/data/panna.xlsx
+++ b/archive/data/panna.xlsx
@@ -13977,7 +13977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1387"/>
+  <dimension ref="A1:M1399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -85665,6 +85665,626 @@
         </is>
       </c>
     </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="F1388" t="inlineStr"/>
+      <c r="G1388" t="inlineStr"/>
+      <c r="H1388" t="inlineStr"/>
+      <c r="I1388" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J1388" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="K1388" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="L1388" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M1388" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>panna_v1</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>44.069925</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>11.282878</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1389" t="inlineStr"/>
+      <c r="J1389" t="inlineStr"/>
+      <c r="K1389" t="inlineStr"/>
+      <c r="L1389" t="inlineStr"/>
+      <c r="M1389" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>panna_v2</t>
+        </is>
+      </c>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>44.056699</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>11.316312</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1390" t="inlineStr"/>
+      <c r="J1390" t="inlineStr"/>
+      <c r="K1390" t="inlineStr"/>
+      <c r="L1390" t="inlineStr"/>
+      <c r="M1390" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>panna_v3</t>
+        </is>
+      </c>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>44.073086</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>11.330343</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1391" t="inlineStr"/>
+      <c r="J1391" t="inlineStr"/>
+      <c r="K1391" t="inlineStr"/>
+      <c r="L1391" t="inlineStr"/>
+      <c r="M1391" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>panna_v4</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>44.092201</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>11.312029</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1392" t="inlineStr"/>
+      <c r="J1392" t="inlineStr"/>
+      <c r="K1392" t="inlineStr"/>
+      <c r="L1392" t="inlineStr"/>
+      <c r="M1392" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>panna_v5</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>44.094786</t>
+        </is>
+      </c>
+      <c r="G1393" t="inlineStr">
+        <is>
+          <t>11.282969</t>
+        </is>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1393" t="inlineStr"/>
+      <c r="J1393" t="inlineStr"/>
+      <c r="K1393" t="inlineStr"/>
+      <c r="L1393" t="inlineStr"/>
+      <c r="M1393" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr"/>
+      <c r="G1394" t="inlineStr"/>
+      <c r="H1394" t="inlineStr"/>
+      <c r="I1394" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J1394" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="K1394" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="L1394" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M1394" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>panna_v1</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>44.069925</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>11.282878</t>
+        </is>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1395" t="inlineStr"/>
+      <c r="J1395" t="inlineStr"/>
+      <c r="K1395" t="inlineStr"/>
+      <c r="L1395" t="inlineStr"/>
+      <c r="M1395" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>panna_v2</t>
+        </is>
+      </c>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>44.056699</t>
+        </is>
+      </c>
+      <c r="G1396" t="inlineStr">
+        <is>
+          <t>11.316312</t>
+        </is>
+      </c>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1396" t="inlineStr"/>
+      <c r="J1396" t="inlineStr"/>
+      <c r="K1396" t="inlineStr"/>
+      <c r="L1396" t="inlineStr"/>
+      <c r="M1396" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>panna_v3</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>44.073086</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>11.330343</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1397" t="inlineStr"/>
+      <c r="J1397" t="inlineStr"/>
+      <c r="K1397" t="inlineStr"/>
+      <c r="L1397" t="inlineStr"/>
+      <c r="M1397" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>panna_v4</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>44.092201</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>11.312029</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1398" t="inlineStr"/>
+      <c r="J1398" t="inlineStr"/>
+      <c r="K1398" t="inlineStr"/>
+      <c r="L1398" t="inlineStr"/>
+      <c r="M1398" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>CUM3</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>panna</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>vertex</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>panna_v5</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>44.094786</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>11.282969</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I1399" t="inlineStr"/>
+      <c r="J1399" t="inlineStr"/>
+      <c r="K1399" t="inlineStr"/>
+      <c r="L1399" t="inlineStr"/>
+      <c r="M1399" t="inlineStr">
+        <is>
+          <t>2026-06-20T19:17:59Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -85676,7 +86296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J232"/>
+  <dimension ref="A1:J234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -97755,6 +98375,110 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-06-20T15:00:00Z</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-06-20T18:00:00Z</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>